<commit_message>
feat: update backlog viewer data and perform repository cleanup
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1265,6 +1265,1051 @@
       </c>
       <c r="J21" s="5" t="inlineStr"/>
       <c r="K21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Cruzamento e Higienizacao de Cartas de Servico (CGE-MS)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>**Descrição**
+Tema de higienização da base de Cartas de Serviço do Portal ms.gov.br. Reduzir duplicidades entre órgãos, padronizar conteúdo e dar ao gestor da CGE-MS uma visão consolidada do que pode ser unificado, mantido ou descartado.
+**Critérios de Aceitação**
+- Snapshot reprodutível da base de cartas extraído por pipeline automatizado.
+- Relatório HTML standalone que mostra clusters de duplicatas, diff entre cópias e KPIs de redução potencial.
+- Documentação mínima (README + plano.md) que permita outro analista rodar o pipeline sem suporte.
+- Aprovação da CGE-MS sobre o formato do relatório.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>cge,cartas-servico,higienizacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Extracao e limpeza de cartas (Postgres -&gt; CSV)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>**Descrição**
+Pipeline de extração que conecta no Postgres (via VPN), aplica JOIN com `gerenciamento_jornada`, limpa HTML/entidades e gera CSV consumível pelas demais etapas. Base reprodutível para todo o cruzamento.
+**Critérios de Aceitação**
+- Comando `run.bat --snapshot` gera CSV em `exports/` sem intervenção manual.
+- HTML e entidades (`&amp;amp;`, `&amp;nbsp;`, etc.) removidos do texto persistido.
+- Conexão configurada via `.env` (sem credenciais no repo).
+- Smoke test (`pytest tests/test_smoke_db.py`) passa com VPN ativa.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>21</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>extracao,limpeza,postgres</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Analise de similaridade e clusterizacao (8 campos ponderados)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>**Descrição**
+Algoritmo de similaridade que pontua pares de cartas com base em 8 campos ponderados (título 25%, descrição 20%, etapas 15%, requisitos 15%, público 10%, nome popular 5%, palavra-chave 5%, tempo 5%) e gera clusters de duplicatas/quase-duplicatas.
+**Critérios de Aceitação**
+- Score composto reproduzível com seed/threshold configuráveis via CLI.
+- Clusters exportados em CSV (`cartas_clusters_resumo.csv`).
+- Diff por cluster (campos iguais vs. campos divergentes) disponível para consumo do relatório.
+- Threshold default 0.65 ajustável via `--threshold`.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>21</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>similaridade,clusters,nlp</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Relatorio HTML standalone para gestor</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>**Descrição**
+Relatório HTML offline para gestor não-técnico (CGE-MS), com KPIs no topo, treemap de proporções, tabela interativa com painel expansivo, diff por cluster, pontuação de qualidade e sugestão de cadastro modelo. Linguagem simples, otimizado para A4.
+**Critérios de Aceitação**
+- Arquivo único, sem dependência de servidor, abre em qualquer navegador.
+- 3 KPIs no topo (serviços ativos, grupos repetidos, potencial de redução).
+- Filtro por órgão + busca por título funcionando client-side.
+- Layout imprimível em A4 sem corte de conteúdo.
+- Validação visual pelo gestor SGD antes do fechamento.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>21</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>relatorio,html,gestao</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Como DBA, quero detectar colunas com HTML/entities (--probe-schema)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>**História do usuário**
+Como DBA, quero identificar colunas da base de Cartas de Serviço que ainda armazenam HTML ou entidades HTML, para priorizar limpeza no banco e evitar reprocessamento no pipeline.
+**Requisitos**
+- Comando `run.bat --probe-schema` varre tabelas-alvo e lista colunas com HTML/entities detectados.
+- Saída legível em terminal + export opcional para CSV.
+**Critérios de Aceitação**
+- Detecta `&lt;tag&gt;`, `&amp;amp;`, `&amp;nbsp;`, `&amp;#xxx;` em colunas TEXT/VARCHAR.
+- Relata nome da coluna, tabela e contagem de ocorrências.
+- Roda sem alterar dado em produção (read-only).</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>22</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>dba,probe-schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Como analista, quero snapshot completo das cartas ativas</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>**História do usuário**
+Como analista da CGE-MS, quero baixar um snapshot completo das cartas de serviço ativas (com etapas, requisitos e órgão), para auditar o estado da base num momento fixo.
+**Requisitos**
+- Snapshot inclui campos: id, título, órgão, descrição, requisitos, público, etapas, prazos, custos, nome popular, palavras-chave, status.
+- Flag `--incluir-inativas` opcional.
+**Critérios de Aceitação**
+- Comando `run.bat --snapshot` gera CSV em `exports/` com nome datado.
+- Execução completa em &lt; 5min para base atual.
+- Sem perda de linhas: contagem CSV = contagem SQL `SELECT count(*)`.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>22</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>snapshot,extracao</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Como gestor, quero detectar duplicatas exatas e similares</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>**História do usuário**
+Como gestor da CGE-MS, quero ver pares e grupos de cartas com conteúdo igual ou muito próximo, para decidir quais unificar e quais manter separadas.
+**Requisitos**
+- Detecção de duplicatas exatas (hash dos campos normalizados).
+- Detecção de similares via score composto (8 campos).
+- Saída em CSV de clusters + insumo para o relatório HTML.
+**Critérios de Aceitação**
+- `run.bat --duplicatas` e `run.bat --similaridade` rodam independentemente.
+- Threshold default 0.65; ajustável via `--threshold`.
+- Cada cluster traz lista de cartas, órgãos envolvidos e score médio.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>23</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>duplicatas,similaridade</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Como gestor, quero pontuacao de qualidade + cadastro modelo sugerido</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>**História do usuário**
+Como gestor da CGE-MS, quero ver, dentro de cada cluster de duplicatas, qual cadastro está mais completo e bem preenchido, para usar como modelo na consolidação.
+**Requisitos**
+- Heurística de qualidade pontua campos preenchidos, tamanho mínimo de descrição, presença de etapas.
+- Cadastro com maior pontuação é destacado no relatório como "sugerido como modelo".
+**Critérios de Aceitação**
+- Pontuação documentada (peso por campo) e reproduzível.
+- Sugestão visível na visualização de cluster do relatório HTML.
+- Empate resolvido por critério estável (ex.: cadastro mais antigo).</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>23</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>qualidade,modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Como gestor, quero relatorio HTML offline com KPIs, treemap e diff</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>**História do usuário**
+Como gestor da CGE-MS, quero abrir um relatório HTML offline com KPIs, treemap, tabela de clusters e diff visual entre cópias, para decidir consolidações sem precisar de suporte técnico.
+**Requisitos**
+- KPIs: serviços ativos, grupos repetidos, potencial de redução.
+- Treemap interativo de proporções.
+- Tabela com painel expansivo por cluster mostrando diff.
+- Filtro por órgão + busca por título.
+- Layout imprimível A4.
+**Critérios de Aceitação**
+- Arquivo único `exports/relatorio.html`, sem CDN externa obrigatória.
+- Abre em Chrome/Edge atualizados sem erro no console.
+- Aprovação visual da SGD antes da entrega à CGE-MS.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>24</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>relatorio,kpi,treemap</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Implementar queries.py com JOIN gerenciamento_jornada</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Implementar `queries.py` com SELECT principal das cartas ativas + JOIN com `gerenciamento_jornada` para trazer etapas. Parametrizar filtro `--incluir-inativas`.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>26</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>sql,queries</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>html_clean.py - strip HTML + decode entities</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Implementar `html_clean.py` com remoção de tags HTML e decodificação de entidades (`html.unescape` + regex). Cobrir casos `&amp;amp;`, `&amp;nbsp;`, `&amp;#xxx;`, comentários e atributos.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>22</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>python,html</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>extracao.py - pipeline fetch + limpeza + CSV</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Implementar `extracao.py` orquestrando fetch via `queries.py`, limpeza via `html_clean.py` e gravação do snapshot CSV em `exports/`. Adicionar log de progresso e contagem final.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>26</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>python,pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>CLI flag --probe-schema em cli.py</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Adicionar flag `--probe-schema` em `cli.py` que invoca rotina de detecção de colunas com HTML/entities e imprime tabela resumida no terminal.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>25</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>cli</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>similaridade.py - score composto 8 campos (titulo 25%, descr 20%...)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Implementar `similaridade.py` com score composto dos 8 campos (título 25%, descrição 20%, etapas 15%, requisitos 15%, público 10%, nome popular 5%, palavra-chave 5%, tempo 5%). Saída: par (id_a, id_b, score).</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>27</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>similaridade,score</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>clusters.py - agrupamento + diff de cluster</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Implementar `clusters.py` agrupando cartas por score acima do threshold (union-find) e gerando, para cada cluster, o diff campo a campo (igual vs. divergente).</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>27</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>clusters,diff</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>CLI flags --threshold e --incluir-inativas</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Expor flags `--threshold &lt;float&gt;` e `--incluir-inativas` em `cli.py`. Validar tipo e faixa (0–1) do threshold.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>27</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>cli</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Heuristica qualidade cadastro + sugestao modelo</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Implementar heurística de qualidade do cadastro (peso por campo preenchido + tamanho mínimo de descrição) e marcar o cadastro de maior pontuação como sugerido como modelo.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>28</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>qualidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>relatorio.html.j2 - 3 KPIs + treemap interativo</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Construir template `templates/relatorio.html.j2` com 3 KPIs no topo e treemap interativo (D3 ou Plotly via CDN local). Renderizar via `relatorio.py`.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>29</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>jinja,html,treemap</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Filtro por orgao + busca por titulo no relatorio</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Adicionar filtro por órgão (select) e busca por título (input) no relatório HTML, com filtragem client-side da tabela de clusters.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>29</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>filtros,ux</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Bloco de diff visual por cluster</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Renderizar bloco de diff visual por cluster: lista de campos iguais (colapsada) e campos divergentes (expandida com lado a lado das cópias).</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>29</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>diff,ux</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Otimizacao A4 para impressao</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Ajustar CSS para impressão A4: `@media print`, quebras de página por cluster, fontes legíveis, ocultar controles interativos.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>29</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>print,css</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>db.py - conexao via .env (python-dotenv + VPN)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Implementar `db.py` carregando credenciais via `python-dotenv` a partir de `.env`. Documentar requisito de VPN ativa.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>22</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>db,env</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>normalize.py - normalizacao de texto</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Implementar `normalize.py` com normalização de texto: lowercase, remoção de acentos, colapso de espaços, strip. Usar nos campos antes da comparação.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>22</v>
+      </c>
+      <c r="G44" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>normalizacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Testes: test_smoke_db.py + test_html_clean.py</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Escrever `tests/test_smoke_db.py` (conexão e SELECT 1 com VPN) e `tests/test_html_clean.py` (cobrindo tags, entidades nomeadas/numéricas, comentários).</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>22</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>testes,pytest</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(backlog): add work items for 5 active SETDIG projects
20 new items (csv_id 115-134) mapped to existing Epic/Feature structure:

- Feature 2.4 Migração EDS→XVia (115-121): FormFlow docs pending,
  handoff with XVia team, gap consolidation across 6 modules
- Feature 2.5 ABEPTIC 2026 / IOSPD (122-126): convalidação evidence
  gaps, Dimensão 1.1 defense, final report submission
- PBI bench-carta (127-129): study done (REMOVER ~0.09%), gerencial
  presentation + event tracking proposal
- PBI prototipo-categorias-ms (130-132): React/Vite prototype ready,
  stakeholder validation + next steps decision
- PBI DS-MS Design System (133-134): levantamento done, catalog to
  vault Obsidian + TFS wiki
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1259,11 +1259,822 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1"/>
-    <row r="18" ht="18" customHeight="1"/>
-    <row r="19" ht="18" customHeight="1"/>
-    <row r="20" ht="18" customHeight="1"/>
-    <row r="21" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" t="n">
+        <v>115</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2.4 Migração EDS → XVia</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Documentação de governança para migração do ecossistema EDS (Control SSO, Admin, Atendimento, Integrador, FormFlow, CMS) para a plataforma XVia. Contrato de 180 dias de migração + 18 meses de operação. 36 serviços MS Digital a migrar + 10 novos autoatendimentos. 465.279+ usuários ativos.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>xvia migracao-eds</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" t="n">
+        <v>116</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Documentação de governança módulo FormFlow</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Como PO, quero ter a documentação de governança do módulo FormFlow completa (visão funcional + documentacao-tecnica.md) para subsidiar o repasse à equipe XVia e reduzir risco operacional na transição. Módulos Control/Admin/Atendimento/Integrador/CMS já possuem doc oficial — FormFlow é o único pendente.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>115</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>8</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>xvia formflow documentacao</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" t="n">
+        <v>117</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Criar documentacao-tecnica.md do módulo FormFlow</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Ler Modulo FormFlow - v1.md e anexos em modulos/formflow/. Consultar manual EDS (https://manuais_ms.gitlab.io/forms/) via Playwright/Firecrawl. Preencher template modulos/TEMPLATE-MODULO.md com as 14+ seções técnicas (stack, fluxos, regras de negócio, integrações, gaps). Seguir padrão dos demais módulos oficiais.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>116</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>xvia formflow</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" t="n">
+        <v>118</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Revisar gaps Modulo FormFlow v1 com equipe XVia</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Identificar e documentar gaps na documentação atual do FormFlow (itens marcados como [a confirmar com EDS] ou 💡 [IA sugere]). Agendar validação com contato técnico EDS/XVia. Registrar veredito por gap no documento.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>116</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>xvia formflow gaps</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" t="n">
+        <v>119</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Validação e handoff dos documentos com fornecedor XVia</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Como PO, quero que todos os documentos de governança dos 6 módulos (Control, Admin, Atendimento, Integrador, FormFlow, CMS) sejam validados pelo novo fornecedor XVia antes do início formal da operação, garantindo entendimento compartilhado das regras de negócio.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>115</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>12</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>xvia handoff validacao</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>120</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Consolidar lista de gaps por módulo (todos os 6)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Varrer os 6 documentos oficiais (modulos/*/Modulo *-v*.md) buscando ocorrências de '[a confirmar com EDS]', '💡 [IA sugere]' e seções incompletas. Gerar planilha de gaps: módulo | seção | gap | status | responsável.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>119</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>4</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>xvia gaps auditoria</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>121</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Agendar reunião de repasse técnico com equipe XVia</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Preparar pauta de repasse com base na lista de gaps (Task #120) e nos documentos oficiais. Contato técnico Integrador: miguel.alencar@extreme.digital. Incluir demo dos fluxos críticos: Control SSO (pré-requisito de todos), Integrador (webhook → API destino), FormFlow (formulários).</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>119</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>xvia handoff reuniao</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>122</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2.5 ABEPTIC 2026 — Avaliação IOSPD</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Participação do MS na avaliação do IOSPD (Índice de Oferta de Serviços Públicos Digitais) — ABEPTIC 2026. Envolve: convalidação das evidências por dimensão, defesa do relatório e submissão final. Referência: Relatório ABEP26.pdf + backlog_convalidacao_v3.csv em projetos/projeto-abep/.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>100</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>abep iospd pesquisa</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>123</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Convalidação IOSPD 2026 — MS</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Como responsável técnico, quero ter todas as dimensões do IOSPD convalidadas com evidências suficientes (✅ ou ⚠️ documentado) para que o MS possa submeter o relatório final ao ABEP 2026 sem pendências críticas.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>122</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>16</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>abep iospd convalidacao</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>124</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Finalizar evidências Dimensão 1.1 para defesa</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Revisar Defesa_Dimensao_1.1.docx em projeto-abep/convalidacao/. Verificar qualificadores ⚠️ (parcial) e ❌ (não atendido) no RELATÓRIO DE CONVALIDAÇÃO - IOSPD 2026.csv. Buscar documentos complementares (decretos, portarias, PTD) para converter ⚠️ em ✅ onde possível.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>123</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="n">
+        <v>4</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>abep dimensao-1.1 evidencias</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>125</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Revisar backlog_convalidacao_v3.csv e fechar gaps abertos</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Abrir backlog_convalidacao_v3.csv, filtrar linhas com status ⚠️ e ❌. Para cada gap: identificar evidência faltante, buscar no site oficial do governo MS ou em decretos/portarias. Usar prompt avalia-pergunta.md para avaliação automatizada via Claude Code.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>123</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="n">
+        <v>6</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>abep convalidacao gaps</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>126</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Submeter relatório final IOSPD ao ABEP 2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Consolidar Relatorio_Convalidacao_MS.html com versão final aprovada. Verificar prazo de submissão ABEPTIC 2026. Exportar evidências no formato exigido. Submeter via canal oficial ABEP.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>123</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>abep submissao relatorio</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>127</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Estudo de Uso do Filtro de Perfil — bench-carta</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Estudo concluído (base 2025): recomendação REMOVER os filtros de Órgão e Perfil do Portal Único. Taxa de uso real do filtro estimada em ~0,091% dos visitantes da home — abaixo do limiar de 2%. Aba Servidor Público: 366 acessos/ano. PBI cobre comunicação e desdobramentos da recomendação.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>101</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="n">
+        <v>6</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>bench-carta filtro-perfil analytics</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>128</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Elaborar apresentação gerencial da recomendação REMOVER</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Preparar apresentação para a gestora (Duda/SGD) com base no relatório docs/estudo-uso-filtro-perfil.md. Incluir: funil de 3 etapas (home → serviço → filtro), KPIs em linguagem simples, comparativo proxy ingênuo (6,05%) vs taxa corrigida (0,091%), recomendação clara REMOVER com justificativa.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>127</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>bench-carta apresentacao gestao</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>129</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Documentar limitação de event tracking e propor instrumentação</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Registrar formalmente a limitação identificada na Fase 1: troca de aba no filtro de Perfil é DOM swap puro — invisível ao Matomo. Redigir proposta de event tracking (ex: dataLayer push ou Custom Dimension Matomo) para medição exata em versão futura. Salvar em docs/ do repo bench-carta.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>127</v>
+      </c>
+      <c r="G31" t="n">
+        <v>3</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>bench-carta event-tracking matomo</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>130</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Prototipagem Seção Categorias Portal MS</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Como PO, quero ter o protótipo da nova seção de categorias do Portal MS validado com as partes interessadas para decidir se avança para implementação. Protótipo React/Vite disponível em projetos/prototipo-categorias-ms/ com responsividade testada (desktop 1280, tablet 639/640, mobile 390).</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>101</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>prototipo categorias portal-ms</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>131</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Apresentar protótipo de categorias para validação com partes interessadas</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Executar o protótipo localmente (npm run dev em prototipo-categorias-ms/). Agendar sessão de validação com SGD/SETDIG. Demonstrar variações responsivas (desktop, tablet, mobile) e o comportamento de expansão de categoria (verify-category-expanded.png). Coletar feedback estruturado.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>130</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="n">
+        <v>2</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>prototipo validacao apresentacao</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>132</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Registrar feedback e definir próximos passos do protótipo</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Após sessão de validação (Task #131): documentar feedback por stakeholder, classificar em: implementar como está / revisar design / descartar. Se aprovado: abrir issue no repositório do Portal Único para implementação. Registrar decisão no Diário de Decisões (skill /decisao).</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>130</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="n">
+        <v>2</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>prototipo feedback decisao</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>133</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Levantamento Material Design System MS (DS-MS)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Levantamento do material existente do Design System do Governo de MS (DS-MS). Artefatos coletados: tokens de cores e tipografia (colors_and_type.css), componentes (components.css), UI kits e assets visuais. Objetivo: ter referência centralizada para uso nos projetos SETDIG.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>101</v>
+      </c>
+      <c r="G35" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="n">
+        <v>4</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>ds-ms design-system</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>134</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Publicar catálogo DS-MS no vault Obsidian e wiki TFS</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Organizar artefatos de projetos/DS-MS Design System/ (colors_and_type.css, components.css, ui_kits/, assets/) em nota estruturada no vault Obsidian (10-conhecimento/setdig/ ou equivalente). Incluir: paleta de cores, tipografia, componentes disponíveis e link para o repositório.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>133</v>
+      </c>
+      <c r="G36" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>ds-ms obsidian catalogo</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update backlog items, sync data files, and add SKILL.md documentation
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1289,14 +1289,11 @@
       <c r="G17" t="n">
         <v>1</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
           <t>xvia migracao-eds</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" t="n">
@@ -1328,7 +1325,6 @@
       <c r="G18" t="n">
         <v>1</v>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
         <v>8</v>
       </c>
@@ -1337,7 +1333,6 @@
           <t>xvia formflow documentacao</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" t="n">
@@ -1369,7 +1364,6 @@
       <c r="G19" t="n">
         <v>1</v>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
         <v>6</v>
       </c>
@@ -1378,7 +1372,6 @@
           <t>xvia formflow</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" t="n">
@@ -1410,7 +1403,6 @@
       <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>3</v>
       </c>
@@ -1419,7 +1411,6 @@
           <t>xvia formflow gaps</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" t="n">
@@ -1451,7 +1442,6 @@
       <c r="G21" t="n">
         <v>1</v>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
         <v>12</v>
       </c>
@@ -1460,7 +1450,6 @@
           <t>xvia handoff validacao</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1492,7 +1481,6 @@
       <c r="G22" t="n">
         <v>1</v>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
         <v>4</v>
       </c>
@@ -1501,7 +1489,6 @@
           <t>xvia gaps auditoria</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1533,7 +1520,6 @@
       <c r="G23" t="n">
         <v>1</v>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
         <v>2</v>
       </c>
@@ -1542,7 +1528,6 @@
           <t>xvia handoff reuniao</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1574,14 +1559,11 @@
       <c r="G24" t="n">
         <v>2</v>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>abep iospd pesquisa</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1613,7 +1595,6 @@
       <c r="G25" t="n">
         <v>2</v>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>16</v>
       </c>
@@ -1622,7 +1603,6 @@
           <t>abep iospd convalidacao</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1654,7 +1634,6 @@
       <c r="G26" t="n">
         <v>2</v>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
         <v>4</v>
       </c>
@@ -1663,7 +1642,6 @@
           <t>abep dimensao-1.1 evidencias</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1695,7 +1673,6 @@
       <c r="G27" t="n">
         <v>2</v>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
         <v>6</v>
       </c>
@@ -1704,7 +1681,6 @@
           <t>abep convalidacao gaps</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1736,7 +1712,6 @@
       <c r="G28" t="n">
         <v>2</v>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
         <v>2</v>
       </c>
@@ -1745,7 +1720,6 @@
           <t>abep submissao relatorio</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1777,7 +1751,6 @@
       <c r="G29" t="n">
         <v>2</v>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
         <v>6</v>
       </c>
@@ -1786,7 +1759,6 @@
           <t>bench-carta filtro-perfil analytics</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1818,7 +1790,6 @@
       <c r="G30" t="n">
         <v>2</v>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
         <v>3</v>
       </c>
@@ -1827,7 +1798,6 @@
           <t>bench-carta apresentacao gestao</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1859,7 +1829,6 @@
       <c r="G31" t="n">
         <v>3</v>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
         <v>2</v>
       </c>
@@ -1868,7 +1837,6 @@
           <t>bench-carta event-tracking matomo</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1900,7 +1868,6 @@
       <c r="G32" t="n">
         <v>2</v>
       </c>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
         <v>5</v>
       </c>
@@ -1909,7 +1876,6 @@
           <t>prototipo categorias portal-ms</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1941,7 +1907,6 @@
       <c r="G33" t="n">
         <v>2</v>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
         <v>2</v>
       </c>
@@ -1950,7 +1915,6 @@
           <t>prototipo validacao apresentacao</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1982,7 +1946,6 @@
       <c r="G34" t="n">
         <v>2</v>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="n">
         <v>2</v>
       </c>
@@ -1991,7 +1954,6 @@
           <t>prototipo feedback decisao</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2023,7 +1985,6 @@
       <c r="G35" t="n">
         <v>3</v>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="n">
         <v>4</v>
       </c>
@@ -2032,7 +1993,6 @@
           <t>ds-ms design-system</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2064,7 +2024,6 @@
       <c r="G36" t="n">
         <v>3</v>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="n">
         <v>3</v>
       </c>
@@ -2073,7 +2032,161 @@
           <t>ds-ms obsidian catalogo</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>135</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Mapeamento Institucional XVia — Órgãos do Governo MS</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>**Historia do usuario**
+Como analista SETDIG, quero ter o cadastro institucional dos 47 orgaos do governo MS (secretario, missao, competencias, estrutura interna) carregado em SQLite e sincronizado com vault Obsidian, para subsidiar analises de governanca digital, relatorios institucionais e o organograma oficial.
+**Requisitos**
+- Pipeline ETL: PDF organograma + Orgaos.csv + Site.csv + scraping /a-secretaria/ -&gt; SQLite
+- Schema com 3 tabelas: secretaria, estrutura_interna, scraping_log
+- Diagrama Mermaid do organograma derivado do Decreto 16.165/2023
+- Notas bidirecionais no vault Obsidian (10-conhecimento/secretarias/)
+**Criterios de Aceitacao**
+- 47 orgaos cadastrados em institucional.db (Fase C concluida)
+- 14 secretarias com dados de scraping coletados (Fase E concluida)
+- Fase F (upsert SQLite com dados de scraping) executada
+- Fase G (organograma.md Mermaid) gerada
+- Fase H (notas Obsidian) publicadas no vault
+- Decisao registrada sobre os 24 orgaos com /a-secretaria/ retornando 404</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>101</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="n">
+        <v>16</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>xvia orgaos-institucionais sqlite obsidian</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>136</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Relatório CGE — análise de 216 erros reportados em serviços do Portal Único</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Processar exports CSV do CGE (2026-05-28T12-28 e 2026-05-28T12-50, 216 linhas cada) com erros reportados pelo cidadao em servicos do Portal Unico MS. Cruzar com Analytics Dashboard.pdf e gerar relatorio consolidado por orgao e tipo de erro.
+Subatividades:
+- Normalizar encoding dos CSVs (cp1252 -&gt; utf-8) e cabecalhos
+- Agrupar por Orgao, Servico, Tipo de Erro
+- Calcular taxas Atendido / Corrigido / Resolucao
+- Cruzar com dados de trafego do dashboard (Matomo idSite=298)
+- Gerar relatorio HTML/markdown com ranking de servicos mais reportados
+- Apresentar a CGE-MS e SGD</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>103</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="n">
+        <v>6</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>relatorio-cge erros portal-unico cge</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>137</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Backlog TFS SETDIG — viewer + skill /tfs para Claude Code</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>**Historia do usuario**
+Como equipe SETDIG, quero ter um backlog TFS local em xlsx com viewer HTML estilo Azure DevOps e skill /tfs para inserir work items via linguagem natural no Claude Code, para reduzir atrito de gestao de backlog sem depender de acesso ao Azure DevOps oficial.
+**Requisitos**
+- backlog.xlsx com schema TFS (csv_id, tipo, titulo, descricao, csv_id_pai, prioridade, sprint, estimativa_horas, tags, ado_id)
+- Conversor xlsx_to_json.py gerando backlog.json + backlog_viewer.html
+- Skill /tfs em ~/.claude/skills/tfs/SKILL.md respeitando hierarquia Epic-&gt;Feature-&gt;PBI-&gt;Task
+- Padroes de descricao por tipo (Epic/Feature, PBI, Task, Bug) conforme TFS.pdf v1 jul/2024
+**Criterios de Aceitacao**
+- Viewer HTML renderiza arvore hierarquica e abre no browser
+- Skill /tfs instalada globalmente e funcional
+- Insercao via linguagem natural mostra previa antes de salvar
+- Apos salvar, xlsx_to_json.py executa e atualiza viewer
+- Campo ado_id permite vincular item local ao Azure DevOps oficial</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>101</v>
+      </c>
+      <c r="G39" t="n">
+        <v>3</v>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="n">
+        <v>8</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>tooling tfs backlog skill claude-code</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(backlog): add 5 PBIs das demandas de 2026-06-11
- 138 Estudo de limite de caracteres das cartas de servico (cruzamento-carta)
- 139 Remocao de itens do portal MS - periodo eleitoral 2026
- 140 Atualizacao do prototipo da carta de servico pos-workshop
- 141 Apresentacao indice ABEP p/ comite
- 142 Apresentacao MAD - acessibilidade & SEO x linguagem simples p/ comite
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2076,7 +2076,6 @@
       <c r="G37" t="n">
         <v>2</v>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="n">
         <v>16</v>
       </c>
@@ -2085,7 +2084,6 @@
           <t>xvia orgaos-institucionais sqlite obsidian</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2124,7 +2122,6 @@
       <c r="G38" t="n">
         <v>2</v>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="n">
         <v>6</v>
       </c>
@@ -2133,7 +2130,6 @@
           <t>relatorio-cge erros portal-unico cge</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2177,7 +2173,6 @@
       <c r="G39" t="n">
         <v>3</v>
       </c>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="n">
         <v>8</v>
       </c>
@@ -2186,7 +2181,201 @@
           <t>tooling tfs backlog skill claude-code</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>138</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Estudo de Limite de Caracteres das Cartas de Servico (cruzamento-carta)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Levantar quantos caracteres a maioria das cartas de servico utiliza para avaliar se faz sentido criar limite de caracteres. Contexto: aproveitar repo C:\Users\Fabio\Documents\SETDIG\2026\projetos\cruzamento-carta e criar nova sessao trazendo este estudo.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>102</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>cartas-servico</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>139</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Remocao de Itens do Portal MS - Periodo Eleitoral 2026</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Remover itens do ms.gov.br referentes ao periodo eleitoral, com base no documento C:\Users\Fabio\Downloads\Alteracoes periodo eleitoral 2026 (1).docx</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>101</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>governanca;eleitoral</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>140</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Atualizacao do Prototipo da Carta de Servico pos-Workshop</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Atualizar prototipo da carta de servico com base no resultado do workshop de ontem. Referencia: C:\Users\Fabio\Downloads\WhatsApp Image 2026-06-11 at 09.28.43.jpeg</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>102</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>cartas-servico;prototipo</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>141</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Apresentacao Indice ABEP p/ Comite</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Consultar vault Obsidian sobre ABEP e montar apresentacao simples (2-3 slides) sobre o indice ABEP para o comite: slide 1 = indice e nossos resultados passados; slide 2 = dimensao da linguagem simples e como avaliam.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>122</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>abep;comite;linguagem-simples</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>142</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Apresentacao MAD - Acessibilidade &amp; SEO x Linguagem Simples p/ Comite</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Mostrar ao comite que acessibilidade e SEO impactam linguagem simples e que a SETDIG mede isso (MAD - Monitor de Acessibilidade Digital). Slide-chave: explicar o que sao os indicadores - Acessibilidade (quao bem o site serve pessoas com deficiencia, ex. 96) e SEO (quao otimizado p/ ser encontrado, ex. 92) e a ponte com linguagem simples. Ref Canva: https://www.canva.com/design/DAHMRauLCl4/LR-D0EouQSTVknqX9tiMdA/edit</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>122</v>
+      </c>
+      <c r="G44" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>mad;acessibilidade;seo;linguagem-simples;comite</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(viewer): status interativo nos work items (A fazer / Em progresso / Finalizado)
- Coluna 'status' no backlog.xlsx (default 'A fazer'; itens novos via /tfs
  podem deixar vazio — conversor normaliza)
- Viewer: dot de status na tree, fracao de progresso em pais (ex. 3/6),
  controle segmentado no painel de detalhe, filtros por status, barra de
  progresso e contadores no header
- Edicao instantanea via localStorage (sem rodar pipeline a cada mudanca);
  overrides sobrevivem a regeneracao do HTML e sao podados quando o xlsx
  ja reflete o valor
- Botao 'Exportar status' baixa status_updates.json; novo apply_status.py
  grava no xlsx e regenera JSON + HTML
- SKILL.md documenta coluna e fluxo de sincronizacao
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -557,6 +557,11 @@
           <t>ado_id</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" t="n">
@@ -596,6 +601,11 @@
           <t>epic,governanca,programa</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" t="n">
@@ -637,6 +647,11 @@
           <t>feature,levantamento,analytics</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" t="n">
@@ -676,6 +691,11 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>feature,cartas-servico,higienizacao</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -730,6 +750,11 @@
           <t>dashboard,matomo,ga4,portal-unico</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" t="n">
@@ -778,6 +803,11 @@
           <t>matomo,top-paginas</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" t="n">
@@ -822,6 +852,11 @@
       <c r="J7" t="inlineStr">
         <is>
           <t>matomo,busca</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -872,6 +907,11 @@
           <t>matomo,transitions,jornada</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" t="n">
@@ -919,6 +959,11 @@
           <t>ga4,ms-digital</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" t="n">
@@ -964,6 +1009,11 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>cartas,ranking,regex</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -1018,6 +1068,11 @@
           <t>cge,cruzamento,similaridade</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" t="n">
@@ -1062,6 +1117,11 @@
       <c r="J12" t="inlineStr">
         <is>
           <t>dba,probe-schema</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -1115,6 +1175,11 @@
           <t>snapshot,extracao,postgres</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" t="n">
@@ -1163,6 +1228,11 @@
           <t>similaridade,clusters</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" t="n">
@@ -1207,6 +1277,11 @@
       <c r="J15" t="inlineStr">
         <is>
           <t>qualidade,modelo</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -1258,6 +1333,11 @@
           <t>relatorio,html,kpi,treemap</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" t="n">
@@ -1294,6 +1374,11 @@
           <t>xvia migracao-eds</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" t="n">
@@ -1333,6 +1418,11 @@
           <t>xvia formflow documentacao</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" t="n">
@@ -1372,6 +1462,11 @@
           <t>xvia formflow</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" t="n">
@@ -1411,6 +1506,11 @@
           <t>xvia formflow gaps</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" t="n">
@@ -1450,6 +1550,11 @@
           <t>xvia handoff validacao</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1489,6 +1594,11 @@
           <t>xvia gaps auditoria</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1528,6 +1638,11 @@
           <t>xvia handoff reuniao</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1564,6 +1679,11 @@
           <t>abep iospd pesquisa</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1603,6 +1723,11 @@
           <t>abep iospd convalidacao</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1642,6 +1767,11 @@
           <t>abep dimensao-1.1 evidencias</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1681,6 +1811,11 @@
           <t>abep convalidacao gaps</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1720,6 +1855,11 @@
           <t>abep submissao relatorio</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1759,6 +1899,11 @@
           <t>bench-carta filtro-perfil analytics</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1798,6 +1943,11 @@
           <t>bench-carta apresentacao gestao</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1837,6 +1987,11 @@
           <t>bench-carta event-tracking matomo</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1876,6 +2031,11 @@
           <t>prototipo categorias portal-ms</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1915,6 +2075,11 @@
           <t>prototipo validacao apresentacao</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1954,6 +2119,11 @@
           <t>prototipo feedback decisao</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1993,6 +2163,11 @@
           <t>ds-ms design-system</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2030,6 +2205,11 @@
       <c r="J36" t="inlineStr">
         <is>
           <t>ds-ms obsidian catalogo</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -2084,6 +2264,11 @@
           <t>xvia orgaos-institucionais sqlite obsidian</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2128,6 +2313,11 @@
       <c r="J38" t="inlineStr">
         <is>
           <t>relatorio-cge erros portal-unico cge</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>A fazer</t>
         </is>
       </c>
     </row>
@@ -2181,6 +2371,11 @@
           <t>tooling tfs backlog skill claude-code</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2212,14 +2407,16 @@
       <c r="G40" t="n">
         <v>2</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>cartas-servico</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2251,14 +2448,16 @@
       <c r="G41" t="n">
         <v>2</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>governanca;eleitoral</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2290,14 +2489,16 @@
       <c r="G42" t="n">
         <v>2</v>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>cartas-servico;prototipo</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2329,14 +2530,16 @@
       <c r="G43" t="n">
         <v>2</v>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>abep;comite;linguagem-simples</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2368,14 +2571,16 @@
       <c r="G44" t="n">
         <v>2</v>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>mad;acessibilidade;seo;linguagem-simples;comite</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>A fazer</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: adiciona PBI 143 - Modelo GCS de governanca de pastas (PoC X-Via)
Ancorado na Feature 115 (2.4 Migracao EDS -> XVia). Regenera backlog.json e viewer (44 itens).
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2579,6 +2579,56 @@
       <c r="L44" t="inlineStr">
         <is>
           <t>A fazer</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>143</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Modelo de Governança de Conteúdo e Estrutura de Projetos (GCS) — padronização de pastas, PoC X-Via</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>**História do usuário**
+Como equipe de projetos da SETDIG, quero um padrão de organização de pastas e artefatos na rede interna (Z:), para localizar documentos rapidamente e eliminar retrabalho e duplicidade.
+**Requisitos**
+- Modelo GCS reaproveitável: princípios, estrutura padrão, regras de nomeação e versionamento
+- Mapa da estrutura atual do X-Via (diagnóstico das dores)
+- Mapa da estrutura ideal (GCS aplicado, cada artefato posicionado)
+- Caso aplicado X-Via com antes x depois e métricas
+- Versões DOCX com timbrado oficial SETDIG
+- Repositório privado versionado no GitHub
+**Critérios de Aceitação**
+- ETP final alcançável em no máximo 3 cliques na estrutura proposta
+- Profundidade máxima de 3 níveis de pasta
+- Zero arquivos duplicados (fonte única da verdade)
+- Nomeação padronizada: minúsculas, prefixo NN-, kebab-case, datas ISO [AAAA-MM-DD]
+- Documentos GCS aprovados e publicados (Markdown + DOCX timbrado)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>115</v>
+      </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>governanca,gcs,xvia,documentacao</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adiciona PBI 144 TODO do dia + 4 tasks (DS-MS, rename projeto, XVia)
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2631,6 +2631,161 @@
           <t>governanca,gcs,xvia,documentacao</t>
         </is>
       </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>144</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Product Backlog Item</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TODO do dia — DS-MS Storybook, revisão Duda, rename projeto, envio XVia (2026-06-22)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>101</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>145</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Deixar Storybook DS-MS fiel à documentação dos componentes</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>144</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>146</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Revisar conteúdo do Storybook que não consegue atualizar (pedido Duda)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>144</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>147</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Renomear projeto "Maturidade Digital" -&gt; "Censo de Serviços Digitais"</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>144</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>148</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Encaminhar documentação/gravação a maycon.lisboa@xvia.com.br e aylime.queiroz@xvia.com.br</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SETDIG</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>144</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>